<commit_message>
adicionando novos casos de teste
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -20,35 +20,26 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
-  <si>
-    <t xml:space="preserve">headerA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">headerB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">headerC</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+  <si>
+    <t xml:space="preserve">hA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hC</t>
   </si>
   <si>
     <t xml:space="preserve">a2</t>
   </si>
   <si>
-    <t xml:space="preserve">b2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c2</t>
-  </si>
-  <si>
     <t xml:space="preserve">a3</t>
   </si>
   <si>
     <t xml:space="preserve">b3</t>
   </si>
   <si>
-    <t xml:space="preserve">c3</t>
-  </si>
-  <si>
     <t xml:space="preserve">a4</t>
   </si>
   <si>
@@ -56,6 +47,27 @@
   </si>
   <si>
     <t xml:space="preserve">c4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d8</t>
   </si>
 </sst>
 </file>
@@ -262,7 +274,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -280,33 +292,56 @@
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="B3" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="C3" s="1"/>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B5" s="0" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C5" s="0" t="s">
         <v>11</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B6" s="0" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C7" s="0" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="D8" s="0" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>